<commit_message>
Add photo-mode actions and default profiles
Extend photo-mode support and add default controller/keymouse profiles. bpsr_controller_helper.py: add new photo-mode camera movement/pan actions, rename some camera/pan action labels, and update CONTROLLER_DIRECTION_ACTION_NAMES and photo-mode links. Add bpsr_controller_helper_config.json with default PlayStation controller and keymouse mappings (photo/fishing mode settings and many action bindings). Also update generated artifacts (bpsr_key_table.xlsx, build/*, dist/*) to reflect these changes.
</commit_message>
<xml_diff>
--- a/bpsr_key_table.xlsx
+++ b/bpsr_key_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\GitHub\BPSRControllerHelper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006C86F4-28F0-4129-B0EC-A7B579507C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{539FB9B3-2F6D-4A8F-95CA-0A384B35BFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="アクション一覧" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3597" uniqueCount="1066">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3597" uniqueCount="1070">
   <si>
     <t>offsets</t>
   </si>
@@ -2632,12 +2632,6 @@
     <t>+0x02305</t>
   </si>
   <si>
-    <t>+0x0230E</t>
-  </si>
-  <si>
-    <t>+0x02323</t>
-  </si>
-  <si>
     <t>+0x02327</t>
   </si>
   <si>
@@ -2647,16 +2641,7 @@
     <t>+0x0237C</t>
   </si>
   <si>
-    <t>撮影モードカメラパン-右</t>
-  </si>
-  <si>
     <t>+0x02396</t>
-  </si>
-  <si>
-    <t>+0x0239F</t>
-  </si>
-  <si>
-    <t>+0x023B4</t>
   </si>
   <si>
     <t>+0x0240D</t>
@@ -3379,6 +3364,340 @@
     <phoneticPr fontId="3"/>
   </si>
   <si>
+    <t>+0x0273A</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x0274F</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>撮影モードカーソル呼出し</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x027B8</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>撮影モードカーソル移動-左右</t>
+    <rPh sb="9" eb="11">
+      <t>イドウ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>撮影モードカーソル移動-上下</t>
+    <rPh sb="9" eb="11">
+      <t>イドウ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>カーソル移動-上下</t>
+    <rPh sb="4" eb="6">
+      <t>イドウ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>カーソル移動-左右</t>
+    <rPh sb="4" eb="6">
+      <t>イドウ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x027FE</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x02821</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x01F40</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x01F63</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモードキャスト/竿を引く</t>
+    <rPh sb="0" eb="1">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>サオ</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>ヒ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード釣り/図鑑</t>
+    <rPh sb="0" eb="1">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>ツリ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>ズカン</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード釣り/研究</t>
+    <rPh sb="0" eb="1">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>ツリ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>ケンキュウ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード釣り餌切替</t>
+    <rPh sb="0" eb="1">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>ツリ</t>
+    </rPh>
+    <rPh sb="7" eb="8">
+      <t>エサ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>キリカエ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード竿切替</t>
+    <rPh sb="0" eb="1">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>サオ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>キリカエ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモードモード/ガイド</t>
+    <rPh sb="0" eb="1">
+      <t>ツ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード設定</t>
+    <rPh sb="0" eb="1">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>セッテイ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモードマウス呼出し</t>
+    <rPh sb="0" eb="1">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>ヨ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>ダ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード竿移動-前</t>
+    <rPh sb="5" eb="6">
+      <t>サオ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>イドウ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>マエ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード竿移動-後</t>
+    <rPh sb="5" eb="6">
+      <t>サオ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>イドウ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>アト</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード竿移動-左</t>
+    <rPh sb="5" eb="6">
+      <t>サオ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>イドウ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>ヒダリ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード竿移動-右</t>
+    <rPh sb="5" eb="6">
+      <t>サオ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>イドウ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>ミギ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード竿移動-前後</t>
+    <rPh sb="5" eb="6">
+      <t>サオ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>イドウ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>ゼンゴ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモード竿移動-左右</t>
+    <rPh sb="5" eb="6">
+      <t>サオ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>イドウ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>サユウ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>釣りモードメニューを閉じる</t>
+    <rPh sb="10" eb="11">
+      <t>ト</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>装備</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>メニューを閉じる</t>
+    <rPh sb="5" eb="6">
+      <t>ト</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x018B1</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x018CB</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x00AC1</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>+0x019C0</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>撮影モードカメラ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>上下</t>
+    </r>
+    <rPh sb="10" eb="11">
+      <t>シタ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>撮影モードカメラ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>左右</t>
+    </r>
+    <rPh sb="9" eb="11">
+      <t>サユウ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -3403,10 +3722,21 @@
         <family val="3"/>
         <charset val="128"/>
       </rPr>
-      <t>上下</t>
+      <t>右</t>
     </r>
-    <rPh sb="12" eb="13">
-      <t>シタ</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>撮影モードカメラパン-上下</t>
+    <rPh sb="11" eb="13">
+      <t>ジョウカ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>撮影モードカメラパン-左右</t>
+    <rPh sb="11" eb="13">
+      <t>サユウ</t>
     </rPh>
     <phoneticPr fontId="3"/>
   </si>
@@ -3418,7 +3748,39 @@
         <family val="3"/>
         <charset val="128"/>
       </rPr>
-      <t>撮影モードカメラパン</t>
+      <t>撮影モードカメラ移動</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>上下</t>
+    </r>
+    <rPh sb="11" eb="13">
+      <t>ジョウカ</t>
+    </rPh>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>撮影モードカメラ移動</t>
     </r>
     <r>
       <rPr>
@@ -3443,273 +3805,19 @@
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>+0x0273A</t>
+    <t>+0x0230E</t>
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>+0x0274F</t>
+    <t>+0x02323</t>
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>撮影モードカーソル呼出し</t>
+    <t>+0x0239F</t>
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>+0x027B8</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>撮影モードカーソル移動-左右</t>
-    <rPh sb="9" eb="11">
-      <t>イドウ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>撮影モードカーソル移動-上下</t>
-    <rPh sb="9" eb="11">
-      <t>イドウ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>カーソル移動-上下</t>
-    <rPh sb="4" eb="6">
-      <t>イドウ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>カーソル移動-左右</t>
-    <rPh sb="4" eb="6">
-      <t>イドウ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>+0x027FE</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>+0x02821</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>+0x01F40</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>+0x01F63</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモードキャスト/竿を引く</t>
-    <rPh sb="0" eb="1">
-      <t>ツ</t>
-    </rPh>
-    <rPh sb="10" eb="11">
-      <t>サオ</t>
-    </rPh>
-    <rPh sb="12" eb="13">
-      <t>ヒ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード釣り/図鑑</t>
-    <rPh sb="0" eb="1">
-      <t>ツ</t>
-    </rPh>
-    <rPh sb="5" eb="6">
-      <t>ツリ</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>ズカン</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード釣り/研究</t>
-    <rPh sb="0" eb="1">
-      <t>ツ</t>
-    </rPh>
-    <rPh sb="5" eb="6">
-      <t>ツリ</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>ケンキュウ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード釣り餌切替</t>
-    <rPh sb="0" eb="1">
-      <t>ツ</t>
-    </rPh>
-    <rPh sb="5" eb="6">
-      <t>ツリ</t>
-    </rPh>
-    <rPh sb="7" eb="8">
-      <t>エサ</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>キリカエ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード竿切替</t>
-    <rPh sb="0" eb="1">
-      <t>ツ</t>
-    </rPh>
-    <rPh sb="5" eb="6">
-      <t>サオ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>キリカエ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモードモード/ガイド</t>
-    <rPh sb="0" eb="1">
-      <t>ツ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード設定</t>
-    <rPh sb="0" eb="1">
-      <t>ツ</t>
-    </rPh>
-    <rPh sb="5" eb="7">
-      <t>セッテイ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモードマウス呼出し</t>
-    <rPh sb="0" eb="1">
-      <t>ツ</t>
-    </rPh>
-    <rPh sb="8" eb="9">
-      <t>ヨ</t>
-    </rPh>
-    <rPh sb="9" eb="10">
-      <t>ダ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード竿移動-前</t>
-    <rPh sb="5" eb="6">
-      <t>サオ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>イドウ</t>
-    </rPh>
-    <rPh sb="9" eb="10">
-      <t>マエ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード竿移動-後</t>
-    <rPh sb="5" eb="6">
-      <t>サオ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>イドウ</t>
-    </rPh>
-    <rPh sb="9" eb="10">
-      <t>アト</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード竿移動-左</t>
-    <rPh sb="5" eb="6">
-      <t>サオ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>イドウ</t>
-    </rPh>
-    <rPh sb="9" eb="10">
-      <t>ヒダリ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード竿移動-右</t>
-    <rPh sb="5" eb="6">
-      <t>サオ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>イドウ</t>
-    </rPh>
-    <rPh sb="9" eb="10">
-      <t>ミギ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード竿移動-前後</t>
-    <rPh sb="5" eb="6">
-      <t>サオ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>イドウ</t>
-    </rPh>
-    <rPh sb="9" eb="11">
-      <t>ゼンゴ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモード竿移動-左右</t>
-    <rPh sb="5" eb="6">
-      <t>サオ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>イドウ</t>
-    </rPh>
-    <rPh sb="9" eb="11">
-      <t>サユウ</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>釣りモードメニューを閉じる</t>
-    <rPh sb="10" eb="11">
-      <t>ト</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>装備</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>メニューを閉じる</t>
-    <rPh sb="5" eb="6">
-      <t>ト</t>
-    </rPh>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>+0x018B1</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>+0x018CB</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>+0x00AC1</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>+0x019C0</t>
+    <t>+0x023B4</t>
     <phoneticPr fontId="3"/>
   </si>
 </sst>
@@ -4255,7 +4363,7 @@
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" ht="14.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>1026</v>
+        <v>1021</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>24</v>
@@ -4267,10 +4375,10 @@
         <v>25</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="14.25" customHeight="1">
@@ -4287,10 +4395,10 @@
         <v>25</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>993</v>
+        <v>988</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -4381,7 +4489,7 @@
         <v>7</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>1019</v>
+        <v>1014</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>9</v>
@@ -4550,7 +4658,7 @@
         <v>663</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>1023</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -5153,7 +5261,7 @@
     </row>
     <row r="53" spans="1:6" ht="14.25" customHeight="1">
       <c r="A53" s="2" t="s">
-        <v>1021</v>
+        <v>1016</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>24</v>
@@ -5165,15 +5273,15 @@
         <v>25</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>996</v>
+        <v>991</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="14.25" customHeight="1">
       <c r="A54" s="2" t="s">
-        <v>1022</v>
+        <v>1017</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>24</v>
@@ -5185,10 +5293,10 @@
         <v>25</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>994</v>
+        <v>989</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -5659,7 +5767,7 @@
         <v>7</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>1018</v>
+        <v>1013</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>9</v>
@@ -6093,7 +6201,7 @@
     </row>
     <row r="100" spans="1:6">
       <c r="A100" s="2" t="s">
-        <v>1064</v>
+        <v>1057</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>7</v>
@@ -6259,7 +6367,7 @@
         <v>7</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="D108" s="2" t="s">
         <v>9</v>
@@ -7017,7 +7125,7 @@
         <v>7</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>1060</v>
+        <v>1053</v>
       </c>
       <c r="D146" s="2" t="s">
         <v>9</v>
@@ -7097,7 +7205,7 @@
         <v>7</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>1016</v>
+        <v>1011</v>
       </c>
       <c r="D150" s="2" t="s">
         <v>9</v>
@@ -7377,7 +7485,7 @@
         <v>7</v>
       </c>
       <c r="C164" s="13" t="s">
-        <v>1012</v>
+        <v>1007</v>
       </c>
       <c r="D164" s="2" t="s">
         <v>9</v>
@@ -7417,7 +7525,7 @@
         <v>7</v>
       </c>
       <c r="C166" s="13" t="s">
-        <v>1013</v>
+        <v>1008</v>
       </c>
       <c r="D166" s="2" t="s">
         <v>9</v>
@@ -7457,7 +7565,7 @@
         <v>7</v>
       </c>
       <c r="C168" s="13" t="s">
-        <v>1014</v>
+        <v>1009</v>
       </c>
       <c r="D168" s="2" t="s">
         <v>9</v>
@@ -7497,7 +7605,7 @@
         <v>7</v>
       </c>
       <c r="C170" s="13" t="s">
-        <v>1015</v>
+        <v>1010</v>
       </c>
       <c r="D170" s="2" t="s">
         <v>9</v>
@@ -8457,7 +8565,7 @@
         <v>7</v>
       </c>
       <c r="C218" s="3" t="s">
-        <v>1061</v>
+        <v>1054</v>
       </c>
       <c r="D218" s="2" t="s">
         <v>9</v>
@@ -8477,7 +8585,7 @@
         <v>24</v>
       </c>
       <c r="C219" s="3" t="s">
-        <v>1061</v>
+        <v>1054</v>
       </c>
       <c r="D219" s="2" t="s">
         <v>25</v>
@@ -8591,7 +8699,7 @@
     </row>
     <row r="225" spans="1:6">
       <c r="A225" s="2" t="s">
-        <v>1062</v>
+        <v>1055</v>
       </c>
       <c r="B225" s="2" t="s">
         <v>7</v>
@@ -8611,7 +8719,7 @@
     </row>
     <row r="226" spans="1:6">
       <c r="A226" s="2" t="s">
-        <v>1063</v>
+        <v>1056</v>
       </c>
       <c r="B226" s="2" t="s">
         <v>24</v>
@@ -8791,7 +8899,7 @@
     </row>
     <row r="235" spans="1:6">
       <c r="A235" s="2" t="s">
-        <v>1065</v>
+        <v>1058</v>
       </c>
       <c r="B235" s="2" t="s">
         <v>7</v>
@@ -9743,7 +9851,7 @@
         <v>25</v>
       </c>
       <c r="E282" s="2" t="s">
-        <v>994</v>
+        <v>989</v>
       </c>
       <c r="F282" s="2" t="s">
         <v>859</v>
@@ -9771,19 +9879,19 @@
     </row>
     <row r="284" spans="1:6">
       <c r="A284" s="2" t="s">
-        <v>1043</v>
+        <v>1036</v>
       </c>
       <c r="B284" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C284" s="14" t="s">
-        <v>1039</v>
+        <v>1032</v>
       </c>
       <c r="D284" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E284" s="2" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="F284" s="2" t="s">
         <v>275</v>
@@ -9811,19 +9919,19 @@
     </row>
     <row r="286" spans="1:6">
       <c r="A286" s="2" t="s">
-        <v>1044</v>
+        <v>1037</v>
       </c>
       <c r="B286" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C286" s="14" t="s">
-        <v>1040</v>
+        <v>1033</v>
       </c>
       <c r="D286" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E286" s="2" t="s">
-        <v>993</v>
+        <v>988</v>
       </c>
       <c r="F286" s="2" t="s">
         <v>862</v>
@@ -9897,7 +10005,7 @@
         <v>7</v>
       </c>
       <c r="C290" s="12" t="s">
-        <v>986</v>
+        <v>981</v>
       </c>
       <c r="D290" s="2" t="s">
         <v>9</v>
@@ -9917,7 +10025,7 @@
         <v>24</v>
       </c>
       <c r="C291" s="12" t="s">
-        <v>986</v>
+        <v>981</v>
       </c>
       <c r="D291" s="2" t="s">
         <v>25</v>
@@ -9937,7 +10045,7 @@
         <v>7</v>
       </c>
       <c r="C292" s="12" t="s">
-        <v>987</v>
+        <v>982</v>
       </c>
       <c r="D292" s="2" t="s">
         <v>9</v>
@@ -9957,7 +10065,7 @@
         <v>24</v>
       </c>
       <c r="C293" s="12" t="s">
-        <v>987</v>
+        <v>982</v>
       </c>
       <c r="D293" s="2" t="s">
         <v>25</v>
@@ -9977,7 +10085,7 @@
         <v>7</v>
       </c>
       <c r="C294" s="12" t="s">
-        <v>988</v>
+        <v>983</v>
       </c>
       <c r="D294" s="2" t="s">
         <v>9</v>
@@ -9997,7 +10105,7 @@
         <v>7</v>
       </c>
       <c r="C295" s="12" t="s">
-        <v>989</v>
+        <v>984</v>
       </c>
       <c r="D295" s="2" t="s">
         <v>9</v>
@@ -10017,7 +10125,7 @@
         <v>24</v>
       </c>
       <c r="C296" s="12" t="s">
-        <v>988</v>
+        <v>983</v>
       </c>
       <c r="D296" s="2" t="s">
         <v>25</v>
@@ -10037,7 +10145,7 @@
         <v>24</v>
       </c>
       <c r="C297" s="12" t="s">
-        <v>989</v>
+        <v>984</v>
       </c>
       <c r="D297" s="2" t="s">
         <v>25</v>
@@ -10057,7 +10165,7 @@
         <v>7</v>
       </c>
       <c r="C298" s="12" t="s">
-        <v>990</v>
+        <v>985</v>
       </c>
       <c r="D298" s="2" t="s">
         <v>9</v>
@@ -10077,7 +10185,7 @@
         <v>24</v>
       </c>
       <c r="C299" s="12" t="s">
-        <v>990</v>
+        <v>985</v>
       </c>
       <c r="D299" s="2" t="s">
         <v>25</v>
@@ -10097,7 +10205,7 @@
         <v>7</v>
       </c>
       <c r="C300" s="12" t="s">
-        <v>991</v>
+        <v>986</v>
       </c>
       <c r="D300" s="2" t="s">
         <v>9</v>
@@ -10117,7 +10225,7 @@
         <v>24</v>
       </c>
       <c r="C301" s="12" t="s">
-        <v>991</v>
+        <v>986</v>
       </c>
       <c r="D301" s="2" t="s">
         <v>25</v>
@@ -10137,7 +10245,7 @@
         <v>7</v>
       </c>
       <c r="C302" s="12" t="s">
-        <v>992</v>
+        <v>987</v>
       </c>
       <c r="D302" s="2" t="s">
         <v>9</v>
@@ -10157,7 +10265,7 @@
         <v>24</v>
       </c>
       <c r="C303" s="12" t="s">
-        <v>992</v>
+        <v>987</v>
       </c>
       <c r="D303" s="2" t="s">
         <v>25</v>
@@ -10257,7 +10365,7 @@
         <v>7</v>
       </c>
       <c r="C308" s="12" t="s">
-        <v>985</v>
+        <v>980</v>
       </c>
       <c r="D308" s="2" t="s">
         <v>9</v>
@@ -10277,7 +10385,7 @@
         <v>24</v>
       </c>
       <c r="C309" s="12" t="s">
-        <v>985</v>
+        <v>980</v>
       </c>
       <c r="D309" s="2" t="s">
         <v>25</v>
@@ -10337,7 +10445,7 @@
         <v>7</v>
       </c>
       <c r="C312" s="13" t="s">
-        <v>1024</v>
+        <v>1019</v>
       </c>
       <c r="D312" s="2" t="s">
         <v>9</v>
@@ -10357,7 +10465,7 @@
         <v>7</v>
       </c>
       <c r="C313" s="2" t="s">
-        <v>1002</v>
+        <v>997</v>
       </c>
       <c r="D313" s="2" t="s">
         <v>9</v>
@@ -10377,7 +10485,7 @@
         <v>7</v>
       </c>
       <c r="C314" s="2" t="s">
-        <v>1004</v>
+        <v>999</v>
       </c>
       <c r="D314" s="2" t="s">
         <v>9</v>
@@ -10451,47 +10559,47 @@
     </row>
     <row r="318" spans="1:6">
       <c r="A318" s="2" t="s">
-        <v>868</v>
+        <v>1066</v>
       </c>
       <c r="B318" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C318" s="2" t="s">
-        <v>28</v>
+      <c r="C318" s="13" t="s">
+        <v>1064</v>
       </c>
       <c r="D318" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E318" s="2" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="F318" s="13" t="s">
-        <v>998</v>
+        <v>993</v>
       </c>
     </row>
     <row r="319" spans="1:6">
       <c r="A319" s="2" t="s">
-        <v>869</v>
+        <v>1067</v>
       </c>
       <c r="B319" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C319" s="2" t="s">
-        <v>28</v>
+      <c r="C319" s="13" t="s">
+        <v>1065</v>
       </c>
       <c r="D319" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E319" s="2" t="s">
+        <v>988</v>
+      </c>
+      <c r="F319" s="2" t="s">
         <v>993</v>
-      </c>
-      <c r="F319" s="2" t="s">
-        <v>998</v>
       </c>
     </row>
     <row r="320" spans="1:6">
       <c r="A320" s="2" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="B320" s="2" t="s">
         <v>7</v>
@@ -10517,7 +10625,7 @@
         <v>7</v>
       </c>
       <c r="C321" s="2" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="D321" s="2" t="s">
         <v>9</v>
@@ -10537,7 +10645,7 @@
         <v>7</v>
       </c>
       <c r="C322" s="13" t="s">
-        <v>1003</v>
+        <v>998</v>
       </c>
       <c r="D322" s="2" t="s">
         <v>9</v>
@@ -10557,7 +10665,7 @@
         <v>7</v>
       </c>
       <c r="C323" s="13" t="s">
-        <v>1005</v>
+        <v>1000</v>
       </c>
       <c r="D323" s="2" t="s">
         <v>9</v>
@@ -10571,7 +10679,7 @@
     </row>
     <row r="324" spans="1:6">
       <c r="A324" s="2" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="B324" s="2" t="s">
         <v>7</v>
@@ -10596,8 +10704,8 @@
       <c r="B325" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C325" s="2" t="s">
-        <v>873</v>
+      <c r="C325" s="13" t="s">
+        <v>1061</v>
       </c>
       <c r="D325" s="2" t="s">
         <v>9</v>
@@ -10611,7 +10719,7 @@
     </row>
     <row r="326" spans="1:6">
       <c r="A326" s="2" t="s">
-        <v>874</v>
+        <v>871</v>
       </c>
       <c r="B326" s="2" t="s">
         <v>7</v>
@@ -10631,42 +10739,42 @@
     </row>
     <row r="327" spans="1:6">
       <c r="A327" s="2" t="s">
-        <v>875</v>
+        <v>1068</v>
       </c>
       <c r="B327" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C327" s="2" t="s">
-        <v>28</v>
+      <c r="C327" s="3" t="s">
+        <v>1062</v>
       </c>
       <c r="D327" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E327" s="2" t="s">
-        <v>996</v>
+        <v>991</v>
       </c>
       <c r="F327" s="2" t="s">
-        <v>998</v>
+        <v>993</v>
       </c>
     </row>
     <row r="328" spans="1:6">
       <c r="A328" s="2" t="s">
-        <v>876</v>
+        <v>1069</v>
       </c>
       <c r="B328" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C328" s="2" t="s">
-        <v>28</v>
+      <c r="C328" s="3" t="s">
+        <v>1063</v>
       </c>
       <c r="D328" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E328" s="2" t="s">
-        <v>994</v>
+        <v>989</v>
       </c>
       <c r="F328" s="2" t="s">
-        <v>998</v>
+        <v>993</v>
       </c>
     </row>
     <row r="329" spans="1:6">
@@ -10677,7 +10785,7 @@
         <v>7</v>
       </c>
       <c r="C329" s="13" t="s">
-        <v>1006</v>
+        <v>1001</v>
       </c>
       <c r="D329" s="2" t="s">
         <v>9</v>
@@ -10697,7 +10805,7 @@
         <v>7</v>
       </c>
       <c r="C330" s="2" t="s">
-        <v>1007</v>
+        <v>1002</v>
       </c>
       <c r="D330" s="2" t="s">
         <v>9</v>
@@ -10717,7 +10825,7 @@
         <v>7</v>
       </c>
       <c r="C331" s="13" t="s">
-        <v>1011</v>
+        <v>1006</v>
       </c>
       <c r="D331" s="2" t="s">
         <v>9</v>
@@ -10731,7 +10839,7 @@
     </row>
     <row r="332" spans="1:6">
       <c r="A332" s="2" t="s">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="B332" s="2" t="s">
         <v>7</v>
@@ -10757,7 +10865,7 @@
         <v>7</v>
       </c>
       <c r="C333" s="13" t="s">
-        <v>1010</v>
+        <v>1005</v>
       </c>
       <c r="D333" s="2" t="s">
         <v>9</v>
@@ -10771,7 +10879,7 @@
     </row>
     <row r="334" spans="1:6">
       <c r="A334" s="2" t="s">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="B334" s="2" t="s">
         <v>7</v>
@@ -10791,47 +10899,47 @@
     </row>
     <row r="335" spans="1:6">
       <c r="A335" s="2" t="s">
-        <v>879</v>
+        <v>874</v>
       </c>
       <c r="B335" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C335" s="2" t="s">
-        <v>1008</v>
+        <v>1003</v>
       </c>
       <c r="D335" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E335" s="2" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="F335" s="2" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
     </row>
     <row r="336" spans="1:6">
       <c r="A336" s="2" t="s">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="B336" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C336" s="2" t="s">
-        <v>1009</v>
+        <v>1004</v>
       </c>
       <c r="D336" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E336" s="2" t="s">
-        <v>993</v>
+        <v>988</v>
       </c>
       <c r="F336" s="2" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
     </row>
     <row r="337" spans="1:6">
       <c r="A337" s="2" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="B337" s="2" t="s">
         <v>7</v>
@@ -10857,7 +10965,7 @@
         <v>7</v>
       </c>
       <c r="C338" s="2" t="s">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="D338" s="2" t="s">
         <v>9</v>
@@ -10877,7 +10985,7 @@
         <v>24</v>
       </c>
       <c r="C339" s="2" t="s">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="D339" s="2" t="s">
         <v>25</v>
@@ -10897,7 +11005,7 @@
         <v>7</v>
       </c>
       <c r="C340" s="2" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="D340" s="2" t="s">
         <v>9</v>
@@ -10917,7 +11025,7 @@
         <v>24</v>
       </c>
       <c r="C341" s="2" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="D341" s="2" t="s">
         <v>25</v>
@@ -10937,7 +11045,7 @@
         <v>7</v>
       </c>
       <c r="C342" s="2" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="D342" s="2" t="s">
         <v>9</v>
@@ -10957,7 +11065,7 @@
         <v>24</v>
       </c>
       <c r="C343" s="2" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="D343" s="2" t="s">
         <v>25</v>
@@ -10977,7 +11085,7 @@
         <v>7</v>
       </c>
       <c r="C344" s="2" t="s">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="D344" s="2" t="s">
         <v>9</v>
@@ -10997,7 +11105,7 @@
         <v>24</v>
       </c>
       <c r="C345" s="2" t="s">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="D345" s="2" t="s">
         <v>25</v>
@@ -11017,7 +11125,7 @@
         <v>7</v>
       </c>
       <c r="C346" s="2" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="D346" s="2" t="s">
         <v>9</v>
@@ -11037,7 +11145,7 @@
         <v>24</v>
       </c>
       <c r="C347" s="2" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="D347" s="2" t="s">
         <v>25</v>
@@ -11057,7 +11165,7 @@
         <v>7</v>
       </c>
       <c r="C348" s="2" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="D348" s="2" t="s">
         <v>9</v>
@@ -11077,7 +11185,7 @@
         <v>24</v>
       </c>
       <c r="C349" s="2" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="D349" s="2" t="s">
         <v>25</v>
@@ -11091,7 +11199,7 @@
     </row>
     <row r="350" spans="1:6">
       <c r="A350" s="2" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
       <c r="B350" s="2" t="s">
         <v>7</v>
@@ -11117,7 +11225,7 @@
         <v>7</v>
       </c>
       <c r="C351" s="3" t="s">
-        <v>1000</v>
+        <v>995</v>
       </c>
       <c r="D351" s="2" t="s">
         <v>9</v>
@@ -11131,7 +11239,7 @@
     </row>
     <row r="352" spans="1:6">
       <c r="A352" s="2" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="B352" s="2" t="s">
         <v>7</v>
@@ -11171,7 +11279,7 @@
     </row>
     <row r="354" spans="1:6">
       <c r="A354" s="2" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="B354" s="2" t="s">
         <v>7</v>
@@ -11217,7 +11325,7 @@
         <v>7</v>
       </c>
       <c r="C356" s="3" t="s">
-        <v>999</v>
+        <v>994</v>
       </c>
       <c r="D356" s="2" t="s">
         <v>9</v>
@@ -11237,7 +11345,7 @@
         <v>24</v>
       </c>
       <c r="C357" s="2" t="s">
-        <v>999</v>
+        <v>994</v>
       </c>
       <c r="D357" s="2" t="s">
         <v>25</v>
@@ -11257,7 +11365,7 @@
         <v>7</v>
       </c>
       <c r="C358" s="3" t="s">
-        <v>1001</v>
+        <v>996</v>
       </c>
       <c r="D358" s="2" t="s">
         <v>9</v>
@@ -11277,7 +11385,7 @@
         <v>24</v>
       </c>
       <c r="C359" s="3" t="s">
-        <v>1001</v>
+        <v>996</v>
       </c>
       <c r="D359" s="2" t="s">
         <v>25</v>
@@ -11291,7 +11399,7 @@
     </row>
     <row r="360" spans="1:6">
       <c r="A360" s="2" t="s">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="B360" s="2" t="s">
         <v>7</v>
@@ -11306,12 +11414,12 @@
         <v>610</v>
       </c>
       <c r="F360" s="2" t="s">
-        <v>892</v>
+        <v>887</v>
       </c>
     </row>
     <row r="361" spans="1:6">
       <c r="A361" s="2" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="B361" s="2" t="s">
         <v>7</v>
@@ -11337,7 +11445,7 @@
         <v>7</v>
       </c>
       <c r="C362" s="2" t="s">
-        <v>1020</v>
+        <v>1015</v>
       </c>
       <c r="D362" s="2" t="s">
         <v>9</v>
@@ -11351,7 +11459,7 @@
     </row>
     <row r="363" spans="1:6">
       <c r="A363" s="2" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="B363" s="2" t="s">
         <v>7</v>
@@ -11371,7 +11479,7 @@
     </row>
     <row r="364" spans="1:6">
       <c r="A364" s="2" t="s">
-        <v>895</v>
+        <v>890</v>
       </c>
       <c r="B364" s="2" t="s">
         <v>7</v>
@@ -11391,47 +11499,47 @@
     </row>
     <row r="365" spans="1:6">
       <c r="A365" s="2" t="s">
-        <v>1033</v>
+        <v>1026</v>
       </c>
       <c r="B365" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C365" s="13" t="s">
-        <v>1031</v>
+        <v>1059</v>
       </c>
       <c r="D365" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E365" s="2" t="s">
-        <v>996</v>
+        <v>991</v>
       </c>
       <c r="F365" s="2" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
     </row>
     <row r="366" spans="1:6">
       <c r="A366" s="2" t="s">
-        <v>1034</v>
+        <v>1027</v>
       </c>
       <c r="B366" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C366" s="13" t="s">
-        <v>1032</v>
+        <v>1060</v>
       </c>
       <c r="D366" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E366" s="2" t="s">
-        <v>994</v>
+        <v>989</v>
       </c>
       <c r="F366" s="2" t="s">
-        <v>897</v>
+        <v>892</v>
       </c>
     </row>
     <row r="367" spans="1:6">
       <c r="A367" s="2" t="s">
-        <v>898</v>
+        <v>893</v>
       </c>
       <c r="B367" s="2" t="s">
         <v>7</v>
@@ -11471,7 +11579,7 @@
     </row>
     <row r="369" spans="1:6">
       <c r="A369" s="2" t="s">
-        <v>899</v>
+        <v>894</v>
       </c>
       <c r="B369" s="2" t="s">
         <v>7</v>
@@ -11511,7 +11619,7 @@
     </row>
     <row r="371" spans="1:6">
       <c r="A371" s="2" t="s">
-        <v>900</v>
+        <v>895</v>
       </c>
       <c r="B371" s="2" t="s">
         <v>7</v>
@@ -11531,13 +11639,13 @@
     </row>
     <row r="372" spans="1:6">
       <c r="A372" s="2" t="s">
-        <v>1036</v>
+        <v>1029</v>
       </c>
       <c r="B372" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C372" s="3" t="s">
-        <v>1035</v>
+        <v>1028</v>
       </c>
       <c r="D372" s="2" t="s">
         <v>25</v>
@@ -11551,7 +11659,7 @@
     </row>
     <row r="373" spans="1:6">
       <c r="A373" s="2" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="B373" s="2" t="s">
         <v>7</v>
@@ -11571,7 +11679,7 @@
     </row>
     <row r="374" spans="1:6">
       <c r="A374" s="2" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
       <c r="B374" s="2" t="s">
         <v>24</v>
@@ -11583,7 +11691,7 @@
         <v>25</v>
       </c>
       <c r="E374" s="2" t="s">
-        <v>994</v>
+        <v>989</v>
       </c>
       <c r="F374" s="2" t="s">
         <v>859</v>
@@ -11591,7 +11699,7 @@
     </row>
     <row r="375" spans="1:6">
       <c r="A375" s="2" t="s">
-        <v>903</v>
+        <v>898</v>
       </c>
       <c r="B375" s="2" t="s">
         <v>7</v>
@@ -11611,19 +11719,19 @@
     </row>
     <row r="376" spans="1:6">
       <c r="A376" s="2" t="s">
-        <v>1041</v>
+        <v>1034</v>
       </c>
       <c r="B376" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C376" s="14" t="s">
-        <v>1038</v>
+        <v>1031</v>
       </c>
       <c r="D376" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E376" s="2" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="F376" s="2" t="s">
         <v>275</v>
@@ -11631,7 +11739,7 @@
     </row>
     <row r="377" spans="1:6">
       <c r="A377" s="2" t="s">
-        <v>904</v>
+        <v>899</v>
       </c>
       <c r="B377" s="2" t="s">
         <v>7</v>
@@ -11651,19 +11759,19 @@
     </row>
     <row r="378" spans="1:6">
       <c r="A378" s="2" t="s">
-        <v>1042</v>
+        <v>1035</v>
       </c>
       <c r="B378" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C378" s="14" t="s">
-        <v>1037</v>
+        <v>1030</v>
       </c>
       <c r="D378" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E378" s="2" t="s">
-        <v>993</v>
+        <v>988</v>
       </c>
       <c r="F378" s="2" t="s">
         <v>862</v>
@@ -11671,7 +11779,7 @@
     </row>
     <row r="379" spans="1:6">
       <c r="A379" s="2" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="B379" s="2" t="s">
         <v>7</v>
@@ -11717,7 +11825,7 @@
         <v>7</v>
       </c>
       <c r="C381" s="2" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="D381" s="2" t="s">
         <v>35</v>
@@ -11737,7 +11845,7 @@
         <v>24</v>
       </c>
       <c r="C382" s="2" t="s">
-        <v>907</v>
+        <v>902</v>
       </c>
       <c r="D382" s="2" t="s">
         <v>25</v>
@@ -11757,7 +11865,7 @@
         <v>24</v>
       </c>
       <c r="C383" s="2" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="D383" s="2" t="s">
         <v>25</v>
@@ -11851,7 +11959,7 @@
     </row>
     <row r="388" spans="1:6">
       <c r="A388" t="s">
-        <v>909</v>
+        <v>904</v>
       </c>
       <c r="B388" t="s">
         <v>7</v>
@@ -11891,13 +11999,13 @@
     </row>
     <row r="390" spans="1:6">
       <c r="A390" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="B390" t="s">
         <v>7</v>
       </c>
       <c r="C390" s="15" t="s">
-        <v>1045</v>
+        <v>1038</v>
       </c>
       <c r="D390" t="s">
         <v>35</v>
@@ -11917,7 +12025,7 @@
         <v>24</v>
       </c>
       <c r="C391" s="15" t="s">
-        <v>1045</v>
+        <v>1038</v>
       </c>
       <c r="D391" t="s">
         <v>25</v>
@@ -11937,7 +12045,7 @@
         <v>7</v>
       </c>
       <c r="C392" s="15" t="s">
-        <v>1046</v>
+        <v>1039</v>
       </c>
       <c r="D392" t="s">
         <v>9</v>
@@ -11957,7 +12065,7 @@
         <v>24</v>
       </c>
       <c r="C393" s="15" t="s">
-        <v>1046</v>
+        <v>1039</v>
       </c>
       <c r="D393" t="s">
         <v>25</v>
@@ -11977,7 +12085,7 @@
         <v>7</v>
       </c>
       <c r="C394" s="15" t="s">
-        <v>1047</v>
+        <v>1040</v>
       </c>
       <c r="D394" t="s">
         <v>9</v>
@@ -11997,7 +12105,7 @@
         <v>24</v>
       </c>
       <c r="C395" s="15" t="s">
-        <v>1047</v>
+        <v>1040</v>
       </c>
       <c r="D395" t="s">
         <v>25</v>
@@ -12017,7 +12125,7 @@
         <v>7</v>
       </c>
       <c r="C396" s="15" t="s">
-        <v>1048</v>
+        <v>1041</v>
       </c>
       <c r="D396" t="s">
         <v>9</v>
@@ -12037,7 +12145,7 @@
         <v>24</v>
       </c>
       <c r="C397" s="15" t="s">
-        <v>1048</v>
+        <v>1041</v>
       </c>
       <c r="D397" t="s">
         <v>25</v>
@@ -12057,7 +12165,7 @@
         <v>7</v>
       </c>
       <c r="C398" s="15" t="s">
-        <v>1049</v>
+        <v>1042</v>
       </c>
       <c r="D398" t="s">
         <v>9</v>
@@ -12077,7 +12185,7 @@
         <v>24</v>
       </c>
       <c r="C399" s="15" t="s">
-        <v>1049</v>
+        <v>1042</v>
       </c>
       <c r="D399" t="s">
         <v>25</v>
@@ -12097,7 +12205,7 @@
         <v>7</v>
       </c>
       <c r="C400" s="15" t="s">
-        <v>1050</v>
+        <v>1043</v>
       </c>
       <c r="D400" t="s">
         <v>9</v>
@@ -12117,7 +12225,7 @@
         <v>24</v>
       </c>
       <c r="C401" s="15" t="s">
-        <v>1050</v>
+        <v>1043</v>
       </c>
       <c r="D401" t="s">
         <v>25</v>
@@ -12137,7 +12245,7 @@
         <v>7</v>
       </c>
       <c r="C402" s="15" t="s">
-        <v>1051</v>
+        <v>1044</v>
       </c>
       <c r="D402" t="s">
         <v>9</v>
@@ -12151,13 +12259,13 @@
     </row>
     <row r="403" spans="1:6">
       <c r="A403" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="B403" t="s">
         <v>24</v>
       </c>
       <c r="C403" s="15" t="s">
-        <v>1051</v>
+        <v>1044</v>
       </c>
       <c r="D403" t="s">
         <v>25</v>
@@ -12166,12 +12274,12 @@
         <v>632</v>
       </c>
       <c r="F403" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
     </row>
     <row r="404" spans="1:6">
       <c r="A404" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
       <c r="B404" t="s">
         <v>7</v>
@@ -12197,7 +12305,7 @@
         <v>7</v>
       </c>
       <c r="C405" s="15" t="s">
-        <v>1052</v>
+        <v>1045</v>
       </c>
       <c r="D405" t="s">
         <v>9</v>
@@ -12217,7 +12325,7 @@
         <v>7</v>
       </c>
       <c r="C406" s="16" t="s">
-        <v>1053</v>
+        <v>1046</v>
       </c>
       <c r="D406" t="s">
         <v>9</v>
@@ -12237,7 +12345,7 @@
         <v>7</v>
       </c>
       <c r="C407" s="16" t="s">
-        <v>1054</v>
+        <v>1047</v>
       </c>
       <c r="D407" t="s">
         <v>9</v>
@@ -12257,7 +12365,7 @@
         <v>7</v>
       </c>
       <c r="C408" s="16" t="s">
-        <v>1055</v>
+        <v>1048</v>
       </c>
       <c r="D408" t="s">
         <v>9</v>
@@ -12271,7 +12379,7 @@
     </row>
     <row r="409" spans="1:6">
       <c r="A409" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="B409" t="s">
         <v>7</v>
@@ -12297,7 +12405,7 @@
         <v>7</v>
       </c>
       <c r="C410" s="16" t="s">
-        <v>1056</v>
+        <v>1049</v>
       </c>
       <c r="D410" t="s">
         <v>9</v>
@@ -12311,7 +12419,7 @@
     </row>
     <row r="411" spans="1:6">
       <c r="A411" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="B411" t="s">
         <v>7</v>
@@ -12331,42 +12439,42 @@
     </row>
     <row r="412" spans="1:6">
       <c r="A412" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="B412" t="s">
         <v>24</v>
       </c>
       <c r="C412" s="16" t="s">
-        <v>1057</v>
+        <v>1050</v>
       </c>
       <c r="D412" t="s">
         <v>25</v>
       </c>
       <c r="E412" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="F412" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
     </row>
     <row r="413" spans="1:6">
       <c r="A413" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
       <c r="B413" t="s">
         <v>24</v>
       </c>
       <c r="C413" s="16" t="s">
-        <v>1058</v>
+        <v>1051</v>
       </c>
       <c r="D413" t="s">
         <v>25</v>
       </c>
       <c r="E413" t="s">
-        <v>993</v>
+        <v>988</v>
       </c>
       <c r="F413" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
     </row>
     <row r="414" spans="1:6">
@@ -12417,7 +12525,7 @@
         <v>7</v>
       </c>
       <c r="C416" s="16" t="s">
-        <v>1059</v>
+        <v>1052</v>
       </c>
       <c r="D416" t="s">
         <v>9</v>
@@ -12437,7 +12545,7 @@
         <v>24</v>
       </c>
       <c r="C417" s="16" t="s">
-        <v>1059</v>
+        <v>1052</v>
       </c>
       <c r="D417" t="s">
         <v>25</v>
@@ -12451,7 +12559,7 @@
     </row>
     <row r="418" spans="1:6">
       <c r="A418" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
       <c r="B418" t="s">
         <v>7</v>
@@ -12491,7 +12599,7 @@
     </row>
     <row r="420" spans="1:6">
       <c r="A420" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="B420" t="s">
         <v>7</v>
@@ -12531,7 +12639,7 @@
     </row>
     <row r="422" spans="1:6">
       <c r="A422" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="B422" t="s">
         <v>7</v>
@@ -12571,7 +12679,7 @@
     </row>
     <row r="424" spans="1:6">
       <c r="A424" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="B424" t="s">
         <v>7</v>
@@ -12611,7 +12719,7 @@
     </row>
     <row r="426" spans="1:6">
       <c r="A426" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
       <c r="B426" t="s">
         <v>7</v>
@@ -12651,7 +12759,7 @@
     </row>
     <row r="428" spans="1:6">
       <c r="A428" t="s">
-        <v>925</v>
+        <v>920</v>
       </c>
       <c r="B428" t="s">
         <v>7</v>
@@ -12691,7 +12799,7 @@
     </row>
     <row r="430" spans="1:6">
       <c r="A430" t="s">
-        <v>926</v>
+        <v>921</v>
       </c>
       <c r="B430" t="s">
         <v>7</v>
@@ -12731,7 +12839,7 @@
     </row>
     <row r="432" spans="1:6">
       <c r="A432" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
       <c r="B432" t="s">
         <v>7</v>
@@ -12771,7 +12879,7 @@
     </row>
     <row r="434" spans="1:6">
       <c r="A434" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
       <c r="B434" t="s">
         <v>7</v>
@@ -12811,7 +12919,7 @@
     </row>
     <row r="436" spans="1:6">
       <c r="A436" t="s">
-        <v>929</v>
+        <v>924</v>
       </c>
       <c r="B436" t="s">
         <v>7</v>
@@ -12851,7 +12959,7 @@
     </row>
     <row r="438" spans="1:6">
       <c r="A438" t="s">
-        <v>930</v>
+        <v>925</v>
       </c>
       <c r="B438" t="s">
         <v>7</v>
@@ -12891,7 +12999,7 @@
     </row>
     <row r="440" spans="1:6">
       <c r="A440" t="s">
-        <v>931</v>
+        <v>926</v>
       </c>
       <c r="B440" t="s">
         <v>7</v>
@@ -12931,7 +13039,7 @@
     </row>
     <row r="442" spans="1:6">
       <c r="A442" t="s">
-        <v>932</v>
+        <v>927</v>
       </c>
       <c r="B442" t="s">
         <v>7</v>
@@ -12971,7 +13079,7 @@
     </row>
     <row r="444" spans="1:6">
       <c r="A444" t="s">
-        <v>933</v>
+        <v>928</v>
       </c>
       <c r="B444" t="s">
         <v>7</v>
@@ -13011,7 +13119,7 @@
     </row>
     <row r="446" spans="1:6">
       <c r="A446" t="s">
-        <v>934</v>
+        <v>929</v>
       </c>
       <c r="B446" t="s">
         <v>7</v>
@@ -13051,7 +13159,7 @@
     </row>
     <row r="448" spans="1:6">
       <c r="A448" t="s">
-        <v>935</v>
+        <v>930</v>
       </c>
       <c r="B448" t="s">
         <v>7</v>
@@ -13091,7 +13199,7 @@
     </row>
     <row r="450" spans="1:6">
       <c r="A450" t="s">
-        <v>936</v>
+        <v>931</v>
       </c>
       <c r="B450" t="s">
         <v>7</v>
@@ -13131,7 +13239,7 @@
     </row>
     <row r="452" spans="1:6">
       <c r="A452" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
       <c r="B452" t="s">
         <v>7</v>
@@ -13171,7 +13279,7 @@
     </row>
     <row r="454" spans="1:6">
       <c r="A454" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
       <c r="B454" t="s">
         <v>7</v>
@@ -13211,7 +13319,7 @@
     </row>
     <row r="456" spans="1:6">
       <c r="A456" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="B456" t="s">
         <v>7</v>
@@ -13251,7 +13359,7 @@
     </row>
     <row r="458" spans="1:6">
       <c r="A458" t="s">
-        <v>940</v>
+        <v>935</v>
       </c>
       <c r="B458" t="s">
         <v>7</v>
@@ -13291,7 +13399,7 @@
     </row>
     <row r="460" spans="1:6">
       <c r="A460" t="s">
-        <v>941</v>
+        <v>936</v>
       </c>
       <c r="B460" t="s">
         <v>7</v>
@@ -13331,7 +13439,7 @@
     </row>
     <row r="462" spans="1:6">
       <c r="A462" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
       <c r="B462" t="s">
         <v>7</v>
@@ -13371,7 +13479,7 @@
     </row>
     <row r="464" spans="1:6">
       <c r="A464" t="s">
-        <v>943</v>
+        <v>938</v>
       </c>
       <c r="B464" t="s">
         <v>7</v>
@@ -13411,7 +13519,7 @@
     </row>
     <row r="466" spans="1:6">
       <c r="A466" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
       <c r="B466" t="s">
         <v>7</v>
@@ -13451,7 +13559,7 @@
     </row>
     <row r="468" spans="1:6">
       <c r="A468" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="B468" t="s">
         <v>7</v>
@@ -13491,7 +13599,7 @@
     </row>
     <row r="470" spans="1:6">
       <c r="A470" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
       <c r="B470" t="s">
         <v>7</v>
@@ -13531,7 +13639,7 @@
     </row>
     <row r="472" spans="1:6">
       <c r="A472" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="B472" t="s">
         <v>7</v>
@@ -13571,7 +13679,7 @@
     </row>
     <row r="474" spans="1:6">
       <c r="A474" t="s">
-        <v>948</v>
+        <v>943</v>
       </c>
       <c r="B474" t="s">
         <v>7</v>
@@ -13611,7 +13719,7 @@
     </row>
     <row r="476" spans="1:6">
       <c r="A476" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
       <c r="B476" t="s">
         <v>7</v>
@@ -13651,7 +13759,7 @@
     </row>
     <row r="478" spans="1:6">
       <c r="A478" t="s">
-        <v>950</v>
+        <v>945</v>
       </c>
       <c r="B478" t="s">
         <v>7</v>
@@ -13691,7 +13799,7 @@
     </row>
     <row r="480" spans="1:6">
       <c r="A480" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
       <c r="B480" t="s">
         <v>7</v>
@@ -13731,7 +13839,7 @@
     </row>
     <row r="482" spans="1:6">
       <c r="A482" t="s">
-        <v>952</v>
+        <v>947</v>
       </c>
       <c r="B482" t="s">
         <v>7</v>
@@ -13771,7 +13879,7 @@
     </row>
     <row r="484" spans="1:6">
       <c r="A484" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
       <c r="B484" t="s">
         <v>7</v>
@@ -13811,7 +13919,7 @@
     </row>
     <row r="486" spans="1:6">
       <c r="A486" t="s">
-        <v>954</v>
+        <v>949</v>
       </c>
       <c r="B486" t="s">
         <v>7</v>
@@ -13851,7 +13959,7 @@
     </row>
     <row r="488" spans="1:6">
       <c r="A488" t="s">
-        <v>955</v>
+        <v>950</v>
       </c>
       <c r="B488" t="s">
         <v>7</v>
@@ -13891,7 +13999,7 @@
     </row>
     <row r="490" spans="1:6">
       <c r="A490" t="s">
-        <v>956</v>
+        <v>951</v>
       </c>
       <c r="B490" t="s">
         <v>7</v>
@@ -13931,7 +14039,7 @@
     </row>
     <row r="492" spans="1:6">
       <c r="A492" t="s">
-        <v>957</v>
+        <v>952</v>
       </c>
       <c r="B492" t="s">
         <v>7</v>
@@ -13971,7 +14079,7 @@
     </row>
     <row r="494" spans="1:6">
       <c r="A494" t="s">
-        <v>958</v>
+        <v>953</v>
       </c>
       <c r="B494" t="s">
         <v>7</v>
@@ -14011,7 +14119,7 @@
     </row>
     <row r="496" spans="1:6">
       <c r="A496" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="B496" t="s">
         <v>7</v>
@@ -14051,7 +14159,7 @@
     </row>
     <row r="498" spans="1:6">
       <c r="A498" t="s">
-        <v>960</v>
+        <v>955</v>
       </c>
       <c r="B498" t="s">
         <v>7</v>
@@ -14091,7 +14199,7 @@
     </row>
     <row r="500" spans="1:6">
       <c r="A500" t="s">
-        <v>961</v>
+        <v>956</v>
       </c>
       <c r="B500" t="s">
         <v>7</v>
@@ -14131,7 +14239,7 @@
     </row>
     <row r="502" spans="1:6">
       <c r="A502" t="s">
-        <v>962</v>
+        <v>957</v>
       </c>
       <c r="B502" t="s">
         <v>7</v>
@@ -14171,7 +14279,7 @@
     </row>
     <row r="504" spans="1:6">
       <c r="A504" t="s">
-        <v>963</v>
+        <v>958</v>
       </c>
       <c r="B504" t="s">
         <v>7</v>
@@ -14211,7 +14319,7 @@
     </row>
     <row r="506" spans="1:6">
       <c r="A506" t="s">
-        <v>964</v>
+        <v>959</v>
       </c>
       <c r="B506" t="s">
         <v>7</v>
@@ -14251,7 +14359,7 @@
     </row>
     <row r="508" spans="1:6">
       <c r="A508" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="B508" t="s">
         <v>7</v>
@@ -14291,7 +14399,7 @@
     </row>
     <row r="510" spans="1:6">
       <c r="A510" t="s">
-        <v>966</v>
+        <v>961</v>
       </c>
       <c r="B510" t="s">
         <v>7</v>
@@ -14331,7 +14439,7 @@
     </row>
     <row r="512" spans="1:6">
       <c r="A512" t="s">
-        <v>967</v>
+        <v>962</v>
       </c>
       <c r="B512" t="s">
         <v>7</v>
@@ -14371,7 +14479,7 @@
     </row>
     <row r="514" spans="1:6">
       <c r="A514" t="s">
-        <v>968</v>
+        <v>963</v>
       </c>
       <c r="B514" t="s">
         <v>7</v>
@@ -14411,7 +14519,7 @@
     </row>
     <row r="516" spans="1:6">
       <c r="A516" t="s">
-        <v>969</v>
+        <v>964</v>
       </c>
       <c r="B516" t="s">
         <v>7</v>
@@ -14451,7 +14559,7 @@
     </row>
     <row r="518" spans="1:6">
       <c r="A518" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="B518" t="s">
         <v>7</v>
@@ -14491,7 +14599,7 @@
     </row>
     <row r="520" spans="1:6">
       <c r="A520" t="s">
-        <v>971</v>
+        <v>966</v>
       </c>
       <c r="B520" t="s">
         <v>7</v>
@@ -14531,7 +14639,7 @@
     </row>
     <row r="522" spans="1:6">
       <c r="A522" t="s">
-        <v>972</v>
+        <v>967</v>
       </c>
       <c r="B522" t="s">
         <v>7</v>
@@ -14571,7 +14679,7 @@
     </row>
     <row r="524" spans="1:6">
       <c r="A524" t="s">
-        <v>973</v>
+        <v>968</v>
       </c>
       <c r="B524" t="s">
         <v>7</v>
@@ -14611,7 +14719,7 @@
     </row>
     <row r="526" spans="1:6">
       <c r="A526" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="B526" t="s">
         <v>7</v>
@@ -14651,7 +14759,7 @@
     </row>
     <row r="528" spans="1:6">
       <c r="A528" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="B528" t="s">
         <v>7</v>
@@ -14691,7 +14799,7 @@
     </row>
     <row r="530" spans="1:6">
       <c r="A530" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
       <c r="B530" t="s">
         <v>7</v>
@@ -14731,7 +14839,7 @@
     </row>
     <row r="532" spans="1:6">
       <c r="A532" t="s">
-        <v>977</v>
+        <v>972</v>
       </c>
       <c r="B532" t="s">
         <v>7</v>
@@ -14771,7 +14879,7 @@
     </row>
     <row r="534" spans="1:6">
       <c r="A534" t="s">
-        <v>978</v>
+        <v>973</v>
       </c>
       <c r="B534" t="s">
         <v>7</v>
@@ -14811,7 +14919,7 @@
     </row>
     <row r="536" spans="1:6">
       <c r="A536" t="s">
-        <v>979</v>
+        <v>974</v>
       </c>
       <c r="B536" t="s">
         <v>7</v>
@@ -14851,7 +14959,7 @@
     </row>
     <row r="538" spans="1:6">
       <c r="A538" t="s">
-        <v>980</v>
+        <v>975</v>
       </c>
       <c r="B538" t="s">
         <v>7</v>
@@ -14931,7 +15039,7 @@
     </row>
     <row r="542" spans="1:6">
       <c r="A542" t="s">
-        <v>981</v>
+        <v>976</v>
       </c>
       <c r="B542" t="s">
         <v>7</v>
@@ -14951,7 +15059,7 @@
     </row>
     <row r="543" spans="1:6">
       <c r="A543" t="s">
-        <v>982</v>
+        <v>977</v>
       </c>
       <c r="B543" t="s">
         <v>7</v>
@@ -14971,7 +15079,7 @@
     </row>
     <row r="544" spans="1:6">
       <c r="A544" t="s">
-        <v>983</v>
+        <v>978</v>
       </c>
       <c r="B544" t="s">
         <v>7</v>
@@ -14991,7 +15099,7 @@
     </row>
     <row r="545" spans="1:6">
       <c r="A545" t="s">
-        <v>984</v>
+        <v>979</v>
       </c>
       <c r="B545" t="s">
         <v>7</v>
@@ -15011,7 +15119,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3"/>
-  <conditionalFormatting sqref="C2:C7 C304:C307 C310:C408 C9:C289 C410:C545">
+  <conditionalFormatting sqref="C2:C7 C304:C307 C9:C289 C410:C545 C310:C408">
     <cfRule type="expression" dxfId="6" priority="5">
       <formula>ISNUMBER(SEARCH("不明",C2))</formula>
     </cfRule>
@@ -15992,7 +16100,7 @@
         <v>35</v>
       </c>
       <c r="B85" s="11" t="s">
-        <v>1025</v>
+        <v>1020</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>609</v>
@@ -16080,7 +16188,7 @@
         <v>624</v>
       </c>
       <c r="B93" s="8" t="s">
-        <v>1027</v>
+        <v>1022</v>
       </c>
       <c r="C93" s="8" t="s">
         <v>611</v>
@@ -16091,7 +16199,7 @@
         <v>624</v>
       </c>
       <c r="B94" s="8" t="s">
-        <v>1028</v>
+        <v>1023</v>
       </c>
       <c r="C94" s="8" t="s">
         <v>613</v>
@@ -16102,7 +16210,7 @@
         <v>624</v>
       </c>
       <c r="B95" s="8" t="s">
-        <v>1029</v>
+        <v>1024</v>
       </c>
       <c r="C95" s="8" t="s">
         <v>615</v>
@@ -16113,7 +16221,7 @@
         <v>624</v>
       </c>
       <c r="B96" s="8" t="s">
-        <v>1030</v>
+        <v>1025</v>
       </c>
       <c r="C96" s="8" t="s">
         <v>617</v>

</xml_diff>